<commit_message>
Kontak bantuan agen ke PIC Agen (kak Virna) di landing, SOP, dan portal
Landing /jadi-agen dan /sop-agen sebelumnya memakai nomor CS umum (Roro). Semua
tombol bantuan di sisi agen kini menuju nomor PIC Agen dan berlabel PIC Agen.
Termasuk tabel pertanyaan terbaru.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pertanyaan-untuk-tim.xlsx
+++ b/docs/pertanyaan-untuk-tim.xlsx
@@ -15,9 +15,9 @@
     <sheet name="Tugas manual" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agen (kak Virna)'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Agen (kak Virna)'!$A$1:$I$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Musafar (pemilik dan tim)'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Keputusan'!$A$1:$G$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Keputusan'!$A$1:$G$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tugas manual'!$A$1:$G$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,15 +729,15 @@
         </is>
       </c>
       <c r="C17" s="9">
-        <f>COUNTA('Agen (kak Virna)'!$C$2:$C$51)</f>
+        <f>COUNTA('Agen (kak Virna)'!$C$2:$C$57)</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>COUNTIF('Agen (kak Virna)'!$G$2:$G$51,"Sudah dijawab")</f>
+        <f>COUNTIF('Agen (kak Virna)'!$G$2:$G$57,"Sudah dijawab")</f>
         <v/>
       </c>
       <c r="E17" s="9">
-        <f>COUNTIF('Agen (kak Virna)'!$G$2:$G$51,"Sebagian")</f>
+        <f>COUNTIF('Agen (kak Virna)'!$G$2:$G$57,"Sebagian")</f>
         <v/>
       </c>
       <c r="F17" s="9">
@@ -787,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -876,7 +876,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Komisi per tingkat untuk paket umroh reguler</t>
+          <t>Tabel komisi per paket (SOP bagian 10 masih kosong: 'Paket Umroh A/B/C Rp ___')</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -886,13 +886,13 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>SOP: Silver Rp1-1,5 jt; Gold Rp1,5-2,5 jt; Platinum Rp2-3 jt. Info ust. Aqlus: Silver 1-1,5 jt; Gold 1,5-2 jt; Platinum 3,5 jt. Gold dan Platinum berbeda: mana yang benar? Berapa untuk Duta Musafar?</t>
+          <t>Sudah ada di surat 035/036/037 untuk 22 keberangkatan Nov 2026 - Mar 2027. Surat untuk periode berikutnya belum ada.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Perlu dicek hukum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Komisi per tingkat untuk paket Super Hemat</t>
+          <t>Bonus closing 5 jamaah Rp 500.000, 10 jamaah Rp 1.500.000, 40 jamaah motor listrik atau tunai. Kalimat 'dalam 1 invoice' maksudnya apa? Dihitung per bulan, per tahun, atau sepanjang waktu?</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Info ust. Aqlus: Silver 500 rb; Gold 1 jt; Platinum 1,5 jt. Tidak disebut di SOP.</t>
+          <t>SOP: bonus hanya berlaku bila agen membawa jamaah secara langsung (bukan dalam periode/dalam 1 invoice), dan nominal tagihan mengikuti harga resmi (bukan promo).</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Tabel komisi per paket (SOP bagian 10 masih kosong: 'Paket Umroh A/B/C Rp ___')</t>
+          <t>Bonus referral agen: tambahan 30% jika agen baru berhasil memberangkatkan jamaah. 30% dari apa (komisi agen baru, komisi pertama saja, atau semua)? Berapa lama berlaku?</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -936,11 +936,15 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr"/>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>SOP: bonus tambahan 30%.</t>
+        </is>
+      </c>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -950,7 +954,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Untuk angka berupa rentang (mis. Silver 1-1,5 jt): apa yang menentukan posisinya? Jenis paket, periode keberangkatan, campaign, promo, atau kebijakan perusahaan?</t>
+          <t>Kapan komisi dibayar? SOP menyebut tiga versi: (1) checklist: setelah pembayaran terverifikasi dan data lengkap, (2) bagian 12: H sampai H+2 jamaah landing, (3) Contoh 2: setelah jamaah berangkat. Mana yang berlaku?</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -960,7 +964,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>SOP: besaran dapat berbeda berdasarkan paket, periode keberangkatan, campaign, promo, kebijakan perusahaan. Aturan pastinya belum ada.</t>
+          <t>SOP: H sampai H+2 jamaah landing. Jawaban kak Virna no. 7 ('saat jamaah berangkat') menjawab paket yang dihitung, dan sejalan dengan komisi layak dibayar saat berangkat. Mohon konfirmasi tanggal bayar.</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr"/>
@@ -976,7 +980,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Paket mana yang termasuk Super Hemat? Ditandai manual atau berdasarkan harga?</t>
+          <t>Apakah agen masih boleh mengajukan penarikan saldo kapan saja? SOP hanya menyebut pembayaran pada H sampai H+2 landing. Berapa minimal?</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -984,11 +988,15 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr"/>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Komisi dibayar saat jamaah berangkat. Penarikan manual kapan saja belum disebut.</t>
+        </is>
+      </c>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -998,7 +1006,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Bonus closing 5 jamaah Rp 500.000, 10 jamaah Rp 1.500.000, 40 jamaah motor listrik atau tunai. Kalimat 'dalam 1 invoice' maksudnya apa? Dihitung per bulan, per tahun, atau sepanjang waktu?</t>
+          <t>Calon agen yang belum bayar biaya registrasi: boleh mendaftarkan lead dan jamaah? (SOP: calon agen belum boleh transaksi atas nama Musafar)</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -1008,7 +1016,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>SOP: bonus hanya berlaku bila agen membawa jamaah secara langsung (bukan dalam periode/dalam 1 invoice), dan nominal tagihan mengikuti harga resmi (bukan promo).</t>
+          <t>Pembayaran dilakukan setelah formulir disetujui. Boleh atau tidaknya mendaftarkan lead sebelum bayar belum disebut.</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr"/>
@@ -1024,7 +1032,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Bonus referral agen: tambahan 30% jika agen baru berhasil memberangkatkan jamaah. 30% dari apa (komisi agen baru, komisi pertama saja, atau semua)? Berapa lama berlaku?</t>
+          <t>Komisi tingkat Duta Musafar: ada atau tidak sampai naik ke Silver? (surat hanya memuat Silver, Gold, Platinum)</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -1032,15 +1040,11 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>SOP: bonus tambahan 30%.</t>
-        </is>
-      </c>
+      <c r="D12" s="13" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Belum</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1054,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Kapan komisi dibayar? SOP menyebut tiga versi: (1) checklist: setelah pembayaran terverifikasi dan data lengkap, (2) bagian 12: H sampai H+2 jamaah landing, (3) Contoh 2: setelah jamaah berangkat. Mana yang berlaku?</t>
+          <t>Jika agen naik tingkat setelah jamaah mendaftar tetapi sebelum jamaah berangkat, komisi jamaah itu memakai tingkat lama atau baru?</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -1058,15 +1062,11 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>SOP 12: H s/d H+2 jamaah landing.</t>
-        </is>
-      </c>
+      <c r="D13" s="13" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Perlu dicek hukum</t>
+          <t>Belum</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Siapa 'pihak berwenang' yang menyetujui komisi (status Approved)?</t>
+          <t>Komisi dibayar saat jamaah berangkat: pembayaran satu kali per keberangkatan (batch), dan tanggal pastinya (H-0 sampai H+2 landing)?</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Apakah agen masih boleh mengajukan penarikan saldo kapan saja? SOP hanya menyebut pembayaran pada H sampai H+2 landing. Berapa minimal?</t>
+          <t>Setelah agen disetujui dan membayar biaya registrasi, kapan status berubah menjadi Agen Aktif dan boleh jualan?</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -1106,15 +1106,11 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>SOP: komisi dibayarkan H s/d H+2; ketentuan tanggal dapat berubah.</t>
-        </is>
-      </c>
+      <c r="D15" s="13" t="inlineStr"/>
       <c r="E15" s="14" t="inlineStr"/>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Belum</t>
         </is>
       </c>
     </row>
@@ -1124,19 +1120,23 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Biaya transfer ditanggung siapa dan berapa?</t>
+          <t>Apakah tingkat bisa turun jika target tidak tercapai? Target minimal 12 jamaah/tahun: apa akibatnya jika tidak tercapai?</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Mendesak</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="inlineStr"/>
+          <t>Penting</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Target minimal 12 jamaah/tahun (SOP; juga disebut kak Virna sebagai ketentuan minimum komisi). Akibat jika tidak tercapai belum disebut.</t>
+        </is>
+      </c>
       <c r="E16" s="14" t="inlineStr"/>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1146,19 +1146,23 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Pajak: PPh dipotong? Apakah wajib NPWP? Berapa persen?</t>
+          <t>Haji khusus: komisi Rp 5.000.000. Apakah paket haji akan dijual lewat sistem ini? Poin 300 per jamaah haji berlaku?</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>Mendesak</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr"/>
+          <t>Penting</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>SOP: Haji khusus Rp5.000.000.</t>
+        </is>
+      </c>
       <c r="E17" s="14" t="inlineStr"/>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1168,19 +1172,23 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Biaya registrasi: bisa dikembalikan jika pendaftaran ditolak atau agen mundur? Boleh dicicil?</t>
+          <t>Komisi untuk anak, bayi, dan peserta non-bed</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Mendesak</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr"/>
+          <t>Penting</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Kak Virna bertanya balik (no. 3): 'Musafar hitungannya gimana?' Perlu jawaban pemilik: apakah bayi dan non-bed dihitung sebagai jamaah untuk komisi, dan berapa?</t>
+        </is>
+      </c>
       <c r="E18" s="14" t="inlineStr"/>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1190,17 +1198,17 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Calon agen yang belum bayar biaya registrasi: boleh mendaftarkan lead dan jamaah? (SOP: calon agen belum boleh transaksi atas nama Musafar)</t>
+          <t>Ketentuan minimum komisi (SOP checklist butir 12): apa maksudnya?</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Mendesak</t>
+          <t>Penting</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>SOP: Calon Agen belum diperbolehkan transaksi atas nama Musafar.</t>
+          <t>12 jamaah per tahun (jawaban kak Virna no. 4). Apakah agen di bawah 12 jamaah/tahun tidak mendapat komisi sama sekali, atau hanya tidak mendapat bonus?</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr"/>
@@ -1216,7 +1224,7 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Apakah tingkat bisa turun jika target tidak tercapai? Target minimal 12 jamaah/tahun: apa akibatnya jika tidak tercapai?</t>
+          <t>Poin: 1 jamaah umroh 100, haji 300, training 20, gathering 30. Nilai penukarannya (merchandise, voucher, cashback umroh, tiket wisata, umroh gratis)?</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -1226,7 +1234,7 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>SOP: target minimal 1 jamaah/bulan atau 12/tahun. Akibatnya belum disebut.</t>
+          <t>SOP: poin bisa ditukar sesuai kebijakan reward tahunan.</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr"/>
@@ -1242,7 +1250,7 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Haji khusus: komisi Rp 5.000.000. Apakah paket haji akan dijual lewat sistem ini? Poin 300 per jamaah haji berlaku?</t>
+          <t>Jika jamaah refund setelah komisi dibayar: dipotong dari komisi berikutnya, dikembalikan agen, atau cara lain? Mana yang utama?</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -1252,7 +1260,7 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>SOP: Haji khusus Rp5.000.000.</t>
+          <t>SOP: salah satu dari ketiganya, perusahaan yang menentukan.</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr"/>
@@ -1268,7 +1276,7 @@
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>Komisi untuk anak, bayi, dan peserta non-bed</t>
+          <t>Diskon pribadi dari agen dikurangi dari fee komisi: dipotong senilai diskon penuh atau persentase?</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -1276,11 +1284,15 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr"/>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>SOP: jika ada diskon akan dikurangi dari fee komisi.</t>
+        </is>
+      </c>
       <c r="E22" s="14" t="inlineStr"/>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1302,7 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Ketentuan minimum komisi (SOP checklist butir 12): apa maksudnya?</t>
+          <t>Komisi memakai tingkat saat jamaah daftar atau saat lunas atau saat berangkat?</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -1298,11 +1310,15 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr"/>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Paket dan kelas yang dihitung: saat jamaah berangkat (no. 7). Tingkat: tingkat agen yang mendaftarkan jamaah (no. 8). Kapan tingkat agen dikunci kalau agen naik tingkat di tengah jalan belum jelas.</t>
+        </is>
+      </c>
       <c r="E23" s="14" t="inlineStr"/>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1328,7 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Poin: 1 jamaah umroh 100, haji 300, training 20, gathering 30. Nilai penukarannya (merchandise, voucher, cashback umroh, tiket wisata, umroh gratis)?</t>
+          <t>Rekening harus atas nama sendiri? Bank apa saja?</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -1322,7 +1338,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>SOP: poin bisa ditukar sesuai kebijakan reward tahunan.</t>
+          <t>SOP: wajib memiliki rekening bank aktif dan nama pemilik rekening.</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr"/>
@@ -1338,7 +1354,7 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Jika jamaah refund setelah komisi dibayar: dipotong dari komisi berikutnya, dikembalikan agen, atau cara lain? Mana yang utama?</t>
+          <t>Berapa lama proses verifikasi dan persetujuan, dan siapa yang menyetujui?</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
@@ -1348,7 +1364,7 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>SOP: salah satu dari ketiganya, perusahaan yang menentukan.</t>
+          <t>SOP: tim Musafar verifikasi data; lama proses tidak disebut.</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr"/>
@@ -1364,7 +1380,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Jika jamaah pindah paket atau tanggal, komisi ikut ke paket baru?</t>
+          <t>Agen Resmi Berkantor vs Agen Individu: apa syarat menjadi Berkantor, dan siapa yang menetapkan?</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1372,11 +1388,15 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr"/>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>SOP: Berkantor boleh memakai identitas Musafar di media sosial; Individu tidak.</t>
+        </is>
+      </c>
       <c r="E26" s="14" t="inlineStr"/>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1406,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Diskon pribadi dari agen dikurangi dari fee komisi: dipotong senilai diskon penuh atau persentase?</t>
+          <t>Agen nonaktif (3 bulan tanpa aktivitas): apa yang dihitung sebagai aktivitas dan bagaimana mengaktifkan kembali?</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -1396,7 +1416,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>SOP: jika ada diskon akan dikurangi dari fee komisi.</t>
+          <t>SOP: nonaktif jika tidak ada aktivitas 3 bulan atau tidak memenuhi administrasi.</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr"/>
@@ -1412,7 +1432,7 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Komisi memakai tingkat saat jamaah daftar atau saat lunas atau saat berangkat?</t>
+          <t>Harga: boleh diturunkan agen?</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -1420,11 +1440,15 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr"/>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Tidak boleh mengubah harga. Diskon pribadi mengurangi fee komisi. Kesepakatan B2B: apa syaratnya?</t>
+        </is>
+      </c>
       <c r="E28" s="14" t="inlineStr"/>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1458,7 @@
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Pembagian 30/70 dan 60/40: persentase dari 'total komisi' yang mana jika kedua agen tingkatnya berbeda?</t>
+          <t>Nomor dan jam layanan PIC Agen</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -1442,11 +1466,15 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr"/>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Virna, Partnership Management Musafar: +62 852-8747-1835. Jam layanan belum disebut.</t>
+        </is>
+      </c>
       <c r="E29" s="14" t="inlineStr"/>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1484,7 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Bukti ke agen: bukti transfer, slip komisi, atau keduanya?</t>
+          <t>Notifikasi untuk agen (disetujui, jamaah daftar, pembayaran masuk, komisi cair): lewat WhatsApp atau email?</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1478,7 +1506,7 @@
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Rekening harus atas nama sendiri? Bank apa saja?</t>
+          <t>Surat komisi untuk keberangkatan setelah Maret 2027 dan Platinum 'Kantor Cabang Resmi': apa syarat menjadi kantor cabang resmi?</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1486,15 +1514,11 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>SOP: wajib memiliki rekening bank aktif dan nama pemilik rekening.</t>
-        </is>
-      </c>
+      <c r="D31" s="13" t="inlineStr"/>
       <c r="E31" s="14" t="inlineStr"/>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Belum</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1528,7 @@
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Berapa lama proses verifikasi dan persetujuan, dan siapa yang menyetujui?</t>
+          <t>Potongan 5%: dari komisi kotor setiap pembayaran? Perlu bukti potong untuk agen?</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1512,15 +1536,11 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
-        <is>
-          <t>SOP: tim Musafar verifikasi data; lama proses tidak disebut.</t>
-        </is>
-      </c>
+      <c r="D32" s="13" t="inlineStr"/>
       <c r="E32" s="14" t="inlineStr"/>
       <c r="F32" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Belum</t>
         </is>
       </c>
     </row>
@@ -1530,17 +1550,17 @@
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Agen Resmi Berkantor vs Agen Individu: apa syarat menjadi Berkantor, dan siapa yang menetapkan?</t>
+          <t>Reward tahunan (Top 10, Top 3, Grand Prize motor target 50 pax, Best Rookie): berapa nominalnya dan kapan diumumkan?</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Penting</t>
+          <t>Nanti</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>SOP: Berkantor boleh memakai identitas Musafar di media sosial; Individu tidak.</t>
+          <t>SOP menyebut jenis hadiah, tanpa nominal.</t>
         </is>
       </c>
       <c r="E33" s="14" t="inlineStr"/>
@@ -1556,17 +1576,17 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Agen nonaktif (3 bulan tanpa aktivitas): apa yang dihitung sebagai aktivitas dan bagaimana mengaktifkan kembali?</t>
+          <t>Komisi yang lama tidak diambil: ada masa kedaluwarsa?</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Penting</t>
+          <t>Nanti</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>SOP: nonaktif jika tidak ada aktivitas 3 bulan atau tidak memenuhi administrasi.</t>
+          <t>Jawaban no. 12: komisi tidak dalam bentuk cash, persentase yang tidak diambil 0%. Tafsir kami: tidak ada kedaluwarsa. Mohon konfirmasi.</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr"/>
@@ -1582,200 +1602,34 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Welcome kit dan perlengkapan: kapan dikirim, siapa menanggung ongkir, ukuran (rompi, koko, abaya) dikumpulkan di mana?</t>
+          <t>Materi pelatihan dan buku panduan yang sudah ada (file)</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>Penting</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="inlineStr"/>
+          <t>Nanti</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>SOP menyebut topik onboarding; file materi belum ada.</t>
+        </is>
+      </c>
       <c r="E35" s="14" t="inlineStr"/>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Harga: boleh diturunkan agen?</t>
-        </is>
-      </c>
-      <c r="C36" s="13" t="inlineStr">
-        <is>
-          <t>Penting</t>
-        </is>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>Tidak boleh mengubah harga. Diskon pribadi mengurangi fee komisi. Kesepakatan B2B: apa syaratnya?</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="inlineStr"/>
-      <c r="F36" s="14" t="inlineStr">
-        <is>
           <t>Sebagian</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Nomor dan jam layanan PIC Agen</t>
-        </is>
-      </c>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>Penting</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>Virna, Partnership Management Musafar: +62 852-8747-1835. Jam layanan belum disebut.</t>
-        </is>
-      </c>
-      <c r="E37" s="14" t="inlineStr"/>
-      <c r="F37" s="14" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Notifikasi untuk agen (disetujui, jamaah daftar, pembayaran masuk, komisi cair): lewat WhatsApp atau email?</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>Penting</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr"/>
-      <c r="E38" s="14" t="inlineStr"/>
-      <c r="F38" s="14" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Reward tahunan (Top 10, Top 3, Grand Prize motor target 50 pax, Best Rookie): berapa nominalnya dan kapan diumumkan?</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>Nanti</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>SOP menyebut jenis hadiah, tanpa nominal.</t>
-        </is>
-      </c>
-      <c r="E39" s="14" t="inlineStr"/>
-      <c r="F39" s="14" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Komisi yang lama tidak diambil: ada masa kedaluwarsa?</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>Nanti</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr"/>
-      <c r="E40" s="14" t="inlineStr"/>
-      <c r="F40" s="14" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>Berapa lama persetujuan konten dan lewat saluran mana?</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>Nanti</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr"/>
-      <c r="E41" s="14" t="inlineStr"/>
-      <c r="F41" s="14" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>Materi pelatihan dan buku panduan yang sudah ada (file)</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>Nanti</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>SOP menyebut topik onboarding; file materi belum ada.</t>
-        </is>
-      </c>
-      <c r="E42" s="14" t="inlineStr"/>
-      <c r="F42" s="14" t="inlineStr">
-        <is>
-          <t>Sebagian</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C42">
+  <conditionalFormatting sqref="C5:C35">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Mendesak"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum,Sebagian,Sudah dijawab,Perlu dicek hukum"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1789,7 +1643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2006,12 +1860,12 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>SOP: target minimal 1 jamaah/bulan atau 12/tahun. Akibatnya belum disebut.</t>
+          <t>Target minimal 12 jamaah/tahun (SOP; juga disebut kak Virna sebagai ketentuan minimum komisi). Akibat jika tidak tercapai belum disebut.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>SOP/AGEN/001</t>
+          <t>Kak Virna</t>
         </is>
       </c>
       <c r="G5" s="14" t="inlineStr">
@@ -2021,7 +1875,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>SOP Target Agen</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr">
@@ -2051,22 +1905,22 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>SOP: Silver Rp1-1,5 jt; Gold Rp1,5-2,5 jt; Platinum Rp2-3 jt. Info ust. Aqlus: Silver 1-1,5 jt; Gold 1,5-2 jt; Platinum 3,5 jt. Gold dan Platinum berbeda: mana yang benar? Berapa untuk Duta Musafar?</t>
+          <t>Pakai angka di surat 035/036/037/MSFR/IX/2026: per tanggal keberangkatan, kelas, dan maskapai (Nov 2026 - Mar 2027). Menggantikan rentang SOP dan info ust. Aqlus.</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>SOP dan Ust. Aqlus</t>
+          <t>Direktur Utama (surat)</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Perlu dicek hukum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>SOP 4e; ust. Aqlus</t>
+          <t>Surat 035-037/MSFR/IX/2026</t>
         </is>
       </c>
       <c r="I6" s="13" t="inlineStr">
@@ -2096,22 +1950,22 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Info ust. Aqlus: Silver 500 rb; Gold 1 jt; Platinum 1,5 jt. Tidak disebut di SOP.</t>
+          <t>Tidak ada paket Super Hemat, hanya Hemat (contoh 10 Jan: Hemat Oman Rp 1.000.000 untuk semua tingkat, sesuai surat).</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Ust. Aqlus</t>
+          <t>Kak Virna</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Ust. Aqlus</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr">
@@ -2139,16 +1993,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr"/>
-      <c r="F8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Sudah ada di surat 035/036/037 untuk 22 keberangkatan Nov 2026 - Mar 2027. Surat untuk periode berikutnya belum ada.</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Direktur Utama (surat)</t>
+        </is>
+      </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>SOP 10</t>
+          <t>Surat 035-037/MSFR/IX/2026</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
@@ -2178,22 +2040,22 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>SOP: besaran dapat berbeda berdasarkan paket, periode keberangkatan, campaign, promo, kebijakan perusahaan. Aturan pastinya belum ada.</t>
+          <t>Ditentukan per tanggal keberangkatan dan kelas, tertulis di surat.</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>SOP/AGEN/001</t>
+          <t>Direktur Utama (surat)</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>Sebagian</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>SOP 10</t>
+          <t>Surat 035-037/MSFR/IX/2026</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
@@ -2221,16 +2083,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada. Hanya kelas Hemat.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
@@ -2303,16 +2173,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna bertanya balik (no. 3): 'Musafar hitungannya gimana?' Perlu jawaban pemilik: apakah bayi dan non-bed dihitung sebagai jamaah untuk komisi, dan berapa?</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I12" s="13" t="inlineStr">
@@ -2385,16 +2263,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>12 jamaah per tahun (jawaban kak Virna no. 4). Apakah agen di bawah 12 jamaah/tahun tidak mendapat komisi sama sekali, atau hanya tidak mendapat bonus?</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>SOP 9</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I14" s="13" t="inlineStr">
@@ -2604,22 +2490,22 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>SOP 12: H s/d H+2 jamaah landing.</t>
+          <t>SOP: H sampai H+2 jamaah landing. Jawaban kak Virna no. 7 ('saat jamaah berangkat') menjawab paket yang dihitung, dan sejalan dengan komisi layak dibayar saat berangkat. Mohon konfirmasi tanggal bayar.</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>SOP/AGEN/001</t>
+          <t>Kak Virna</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>Perlu dicek hukum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>SOP 9, 12, 23</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
@@ -2647,16 +2533,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr"/>
-      <c r="F20" s="14" t="inlineStr"/>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Manajemen dan finance.</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>SOP 11</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
@@ -2774,16 +2668,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr"/>
-      <c r="F23" s="14" t="inlineStr"/>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Ya, komisi mengikuti paket baru.</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
@@ -2856,16 +2758,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr"/>
-      <c r="F25" s="14" t="inlineStr"/>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Paket dan kelas yang dihitung: saat jamaah berangkat (no. 7). Tingkat: tingkat agen yang mendaftarkan jamaah (no. 8). Kapan tingkat agen dikunci kalau agen naik tingkat di tengah jalan belum jelas.</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
@@ -3028,16 +2938,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr"/>
-      <c r="F29" s="14" t="inlineStr"/>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Total komisi mengikuti tingkat agen yang mendaftarkan jamaah (agen Gold = komisi Gold), lalu dibagi 30/70 atau 60/40.</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t>SOP 6</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I29" s="13" t="inlineStr">
@@ -3067,12 +2985,12 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>SOP: komisi dibayarkan H s/d H+2; ketentuan tanggal dapat berubah.</t>
+          <t>Komisi dibayar saat jamaah berangkat. Penarikan manual kapan saja belum disebut.</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t>SOP/AGEN/001</t>
+          <t>Kak Virna</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -3082,7 +3000,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>SOP 12</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
@@ -3110,16 +3028,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr"/>
-      <c r="F31" s="14" t="inlineStr"/>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Musafar.</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I31" s="13" t="inlineStr">
@@ -3147,16 +3073,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr"/>
-      <c r="F32" s="14" t="inlineStr"/>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Dipotong 5%. NPWP tidak wajib, NIK wajib.</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I32" s="13" t="inlineStr">
@@ -3184,16 +3118,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr"/>
-      <c r="F33" s="14" t="inlineStr"/>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Bukti transfer.</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I33" s="13" t="inlineStr">
@@ -3266,16 +3208,24 @@
           <t>Nanti</t>
         </is>
       </c>
-      <c r="E35" s="14" t="inlineStr"/>
-      <c r="F35" s="14" t="inlineStr"/>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Jawaban no. 12: komisi tidak dalam bentuk cash, persentase yang tidak diambil 0%. Tafsir kami: tidak ada kedaluwarsa. Mohon konfirmasi.</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sebagian</t>
         </is>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I35" s="13" t="inlineStr">
@@ -3393,16 +3343,24 @@
           <t>Mendesak</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr"/>
-      <c r="F38" s="14" t="inlineStr"/>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>Dibayar setelah formulir disetujui. Jika agen mundur, biaya hangus karena ditukar dengan perlengkapan dan welcome kit. Cicilan tidak disarankan.</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I38" s="13" t="inlineStr">
@@ -3432,12 +3390,12 @@
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>SOP: Calon Agen belum diperbolehkan transaksi atas nama Musafar.</t>
+          <t>Pembayaran dilakukan setelah formulir disetujui. Boleh atau tidaknya mendaftarkan lead sebelum bayar belum disebut.</t>
         </is>
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>SOP/AGEN/001</t>
+          <t>Kak Virna</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
@@ -3447,7 +3405,7 @@
       </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
-          <t>SOP 5</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I39" s="13" t="inlineStr">
@@ -3655,16 +3613,24 @@
           <t>Penting</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr"/>
-      <c r="F44" s="14" t="inlineStr"/>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Dikirim akhir Oktober 2026 (insyaAllah). Ongkir ditanggung agen. Form ukuran dikirim kak Virna setelah daftar.</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>SOP 4b</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
@@ -3782,16 +3748,24 @@
           <t>Nanti</t>
         </is>
       </c>
-      <c r="E47" s="14" t="inlineStr"/>
-      <c r="F47" s="14" t="inlineStr"/>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Dikirim ke WhatsApp PIC Agen, selesai kurang dari 24 jam.</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Sudah dijawab</t>
         </is>
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>SOP 5c</t>
+          <t>Kak Virna 7 Okt</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
@@ -3972,14 +3946,236 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="13" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>Komisi tingkat Duta Musafar: ada atau tidak sampai naik ke Silver? (surat hanya memuat Silver, Gold, Platinum)</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>Mendesak</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr"/>
+      <c r="F52" s="14" t="inlineStr"/>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>Surat 035-037/MSFR/IX/2026</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>Isi sel Duta di Komisi Agen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>Surat komisi untuk keberangkatan setelah Maret 2027 dan Platinum 'Kantor Cabang Resmi': apa syarat menjadi kantor cabang resmi?</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Penting</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr"/>
+      <c r="F53" s="14" t="inlineStr"/>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H53" s="13" t="inlineStr">
+        <is>
+          <t>Surat 035-037/MSFR/IX/2026</t>
+        </is>
+      </c>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>Tabel komisi periode berikutnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Jika agen naik tingkat setelah jamaah mendaftar tetapi sebelum jamaah berangkat, komisi jamaah itu memakai tingkat lama atau baru?</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Mendesak</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr"/>
+      <c r="F54" s="14" t="inlineStr"/>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>Kak Virna 7 Okt</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>Aturan tingkat komisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Potongan 5%: dari komisi kotor setiap pembayaran? Perlu bukti potong untuk agen?</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Penting</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr"/>
+      <c r="F55" s="14" t="inlineStr"/>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Kak Virna 7 Okt</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>Slip komisi dan pajak</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Komisi dibayar saat jamaah berangkat: pembayaran satu kali per keberangkatan (batch), dan tanggal pastinya (H-0 sampai H+2 landing)?</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Mendesak</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr"/>
+      <c r="F56" s="14" t="inlineStr"/>
+      <c r="G56" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>Kak Virna 7 Okt</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>Jadwal bayar komisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Pertanyaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Setelah agen disetujui dan membayar biaya registrasi, kapan status berubah menjadi Agen Aktif dan boleh jualan?</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Mendesak</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr"/>
+      <c r="F57" s="14" t="inlineStr"/>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>Kak Virna 7 Okt</t>
+        </is>
+      </c>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>Gerbang akses portal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
-  <conditionalFormatting sqref="D2:D51">
+  <autoFilter ref="A1:I57"/>
+  <conditionalFormatting sqref="D2:D57">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Mendesak"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G51">
+  <conditionalFormatting sqref="G2:G57">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"Sudah dijawab"</formula>
     </cfRule>
@@ -3988,10 +4184,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum,Sebagian,Sudah dijawab,Perlu dicek hukum"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Mendesak,Penting,Nanti"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6047,7 +6243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6178,79 +6374,211 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
+          <t>Tabel komisi</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Komisi per keberangkatan, kelas, dan tingkat sesuai surat 035/036/037/MSFR/IX/2026; tidak ada Super Hemat</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Direktur Utama; kak Virna</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Menggantikan komisi flat Rp 1,5 jt</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Sudah di sistem (Komisi Agen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Waktu bayar komisi</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Komisi mengikuti paket yang berangkat; layak dibayar saat jamaah berangkat (SOP: H sampai H+2); disetujui manajemen dan finance</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Total komisi mengikuti tingkat agen yang mendaftarkan jamaah</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Ya: status komisi</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Menunggu dibangun</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Pajak komisi</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Dipotong 5%; NPWP tidak wajib, NIK wajib; biaya transfer ditanggung Musafar; bukti: bukti transfer</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Menunggu dibangun</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Biaya registrasi agen</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Dibayar setelah formulir disetujui; hangus jika agen mundur; cicilan tidak disarankan</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Ditukar perlengkapan dan welcome kit</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Ya: urutan alur</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Menunggu dibangun</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Persetujuan konten</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Lewat WhatsApp PIC Agen, kurang dari 24 jam</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Kak Virna</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Sudah dicatat</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
           <t>Pelacakan (cookie)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Sementara: tag pelacakan tidak jalan di halaman bertoken. Banner persetujuan belum diputuskan</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Pemilik</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Minimum yang aman dulu</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Mungkin</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Menunggu keputusan banner</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="n"/>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="14" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="n"/>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="14" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n"/>
@@ -6477,10 +6805,55 @@
       <c r="F34" s="14" t="n"/>
       <c r="G34" s="14" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="14" t="n"/>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="n"/>
+      <c r="B36" s="14" t="n"/>
+      <c r="C36" s="14" t="n"/>
+      <c r="D36" s="14" t="n"/>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="14" t="n"/>
+      <c r="G36" s="14" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+      <c r="G37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="n"/>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+      <c r="G38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="14" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G34"/>
+  <autoFilter ref="A1:G39"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Menunggu,Menunggu tabel,Menunggu keputusan banner,Sedang dikerjakan,Sudah di sistem,Tidak perlu"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>